<commit_message>
improved phytoseilus bulk to display day and monthly data
</commit_message>
<xml_diff>
--- a/exports/QC_Database.xlsx
+++ b/exports/QC_Database.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T210"/>
+  <dimension ref="A1:T246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2117,14 +2117,30 @@
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2171,14 +2187,30 @@
       </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2225,14 +2257,30 @@
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2279,14 +2327,30 @@
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2333,14 +2397,30 @@
       </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
-      <c r="T35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2387,14 +2467,30 @@
       </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3987,14 +4083,30 @@
       </c>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
-      <c r="R68" t="inlineStr"/>
-      <c r="S68" t="inlineStr"/>
-      <c r="T68" t="inlineStr"/>
+      <c r="M68" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" t="n">
+        <v>0</v>
+      </c>
+      <c r="P68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>0</v>
+      </c>
+      <c r="R68" t="n">
+        <v>0</v>
+      </c>
+      <c r="S68" t="n">
+        <v>0</v>
+      </c>
+      <c r="T68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4037,14 +4149,30 @@
       </c>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
-      <c r="T69" t="inlineStr"/>
+      <c r="M69" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>0</v>
+      </c>
+      <c r="R69" t="n">
+        <v>0</v>
+      </c>
+      <c r="S69" t="n">
+        <v>0</v>
+      </c>
+      <c r="T69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -4087,14 +4215,30 @@
       </c>
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
-      <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
-      <c r="T70" t="inlineStr"/>
+      <c r="M70" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0</v>
+      </c>
+      <c r="P70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R70" t="n">
+        <v>0</v>
+      </c>
+      <c r="S70" t="n">
+        <v>0</v>
+      </c>
+      <c r="T70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -4137,14 +4281,30 @@
       </c>
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr"/>
-      <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
-      <c r="T71" t="inlineStr"/>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>0</v>
+      </c>
+      <c r="R71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S71" t="n">
+        <v>0</v>
+      </c>
+      <c r="T71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -4187,14 +4347,30 @@
       </c>
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
-      <c r="T72" t="inlineStr"/>
+      <c r="M72" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0</v>
+      </c>
+      <c r="P72" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>0</v>
+      </c>
+      <c r="R72" t="n">
+        <v>0</v>
+      </c>
+      <c r="S72" t="n">
+        <v>0</v>
+      </c>
+      <c r="T72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4237,14 +4413,30 @@
       </c>
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
-      <c r="P73" t="inlineStr"/>
-      <c r="Q73" t="inlineStr"/>
-      <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr"/>
-      <c r="T73" t="inlineStr"/>
+      <c r="M73" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>0</v>
+      </c>
+      <c r="R73" t="n">
+        <v>0</v>
+      </c>
+      <c r="S73" t="n">
+        <v>0</v>
+      </c>
+      <c r="T73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -4287,14 +4479,30 @@
       </c>
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
-      <c r="P74" t="inlineStr"/>
-      <c r="Q74" t="inlineStr"/>
-      <c r="R74" t="inlineStr"/>
-      <c r="S74" t="inlineStr"/>
-      <c r="T74" t="inlineStr"/>
+      <c r="M74" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" t="n">
+        <v>0</v>
+      </c>
+      <c r="P74" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>0</v>
+      </c>
+      <c r="R74" t="n">
+        <v>0</v>
+      </c>
+      <c r="S74" t="n">
+        <v>0</v>
+      </c>
+      <c r="T74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -4337,14 +4545,30 @@
       </c>
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
-      <c r="P75" t="inlineStr"/>
-      <c r="Q75" t="inlineStr"/>
-      <c r="R75" t="inlineStr"/>
-      <c r="S75" t="inlineStr"/>
-      <c r="T75" t="inlineStr"/>
+      <c r="M75" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0</v>
+      </c>
+      <c r="R75" t="n">
+        <v>0</v>
+      </c>
+      <c r="S75" t="n">
+        <v>0</v>
+      </c>
+      <c r="T75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -4387,14 +4611,30 @@
       </c>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
-      <c r="P76" t="inlineStr"/>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr"/>
-      <c r="S76" t="inlineStr"/>
-      <c r="T76" t="inlineStr"/>
+      <c r="M76" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>0</v>
+      </c>
+      <c r="R76" t="n">
+        <v>0</v>
+      </c>
+      <c r="S76" t="n">
+        <v>0</v>
+      </c>
+      <c r="T76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -4437,14 +4677,30 @@
       </c>
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
-      <c r="P77" t="inlineStr"/>
-      <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr"/>
-      <c r="S77" t="inlineStr"/>
-      <c r="T77" t="inlineStr"/>
+      <c r="M77" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>0</v>
+      </c>
+      <c r="R77" t="n">
+        <v>0</v>
+      </c>
+      <c r="S77" t="n">
+        <v>0</v>
+      </c>
+      <c r="T77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -4487,14 +4743,30 @@
       </c>
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
-      <c r="P78" t="inlineStr"/>
-      <c r="Q78" t="inlineStr"/>
-      <c r="R78" t="inlineStr"/>
-      <c r="S78" t="inlineStr"/>
-      <c r="T78" t="inlineStr"/>
+      <c r="M78" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>0</v>
+      </c>
+      <c r="R78" t="n">
+        <v>0</v>
+      </c>
+      <c r="S78" t="n">
+        <v>0</v>
+      </c>
+      <c r="T78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -4537,14 +4809,30 @@
       </c>
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
-      <c r="P79" t="inlineStr"/>
-      <c r="Q79" t="inlineStr"/>
-      <c r="R79" t="inlineStr"/>
-      <c r="S79" t="inlineStr"/>
-      <c r="T79" t="inlineStr"/>
+      <c r="M79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>0</v>
+      </c>
+      <c r="R79" t="n">
+        <v>0</v>
+      </c>
+      <c r="S79" t="n">
+        <v>0</v>
+      </c>
+      <c r="T79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -4587,14 +4875,30 @@
       </c>
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
-      <c r="P80" t="inlineStr"/>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
-      <c r="S80" t="inlineStr"/>
-      <c r="T80" t="inlineStr"/>
+      <c r="M80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0</v>
+      </c>
+      <c r="S80" t="n">
+        <v>0</v>
+      </c>
+      <c r="T80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -4637,14 +4941,30 @@
       </c>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
-      <c r="P81" t="inlineStr"/>
-      <c r="Q81" t="inlineStr"/>
-      <c r="R81" t="inlineStr"/>
-      <c r="S81" t="inlineStr"/>
-      <c r="T81" t="inlineStr"/>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0</v>
+      </c>
+      <c r="P81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>0</v>
+      </c>
+      <c r="R81" t="n">
+        <v>0</v>
+      </c>
+      <c r="S81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4687,14 +5007,30 @@
       </c>
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
-      <c r="P82" t="inlineStr"/>
-      <c r="Q82" t="inlineStr"/>
-      <c r="R82" t="inlineStr"/>
-      <c r="S82" t="inlineStr"/>
-      <c r="T82" t="inlineStr"/>
+      <c r="M82" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0</v>
+      </c>
+      <c r="P82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>0</v>
+      </c>
+      <c r="R82" t="n">
+        <v>0</v>
+      </c>
+      <c r="S82" t="n">
+        <v>0</v>
+      </c>
+      <c r="T82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -8747,14 +9083,30 @@
         </is>
       </c>
       <c r="L162" t="inlineStr"/>
-      <c r="M162" t="inlineStr"/>
-      <c r="N162" t="inlineStr"/>
-      <c r="O162" t="inlineStr"/>
-      <c r="P162" t="inlineStr"/>
-      <c r="Q162" t="inlineStr"/>
-      <c r="R162" t="inlineStr"/>
-      <c r="S162" t="inlineStr"/>
-      <c r="T162" t="inlineStr"/>
+      <c r="M162" t="n">
+        <v>0</v>
+      </c>
+      <c r="N162" t="n">
+        <v>0</v>
+      </c>
+      <c r="O162" t="n">
+        <v>0</v>
+      </c>
+      <c r="P162" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>0</v>
+      </c>
+      <c r="R162" t="n">
+        <v>0</v>
+      </c>
+      <c r="S162" t="n">
+        <v>0</v>
+      </c>
+      <c r="T162" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -11686,6 +12038,2530 @@
         <v>0</v>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>212</v>
+      </c>
+      <c r="B211" t="n">
+        <v>38</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Phytoseiulus</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F211" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="G211" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>1,000,000</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Mites to phytoseiulus Ratio was balanced</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>1,000,000</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Biobest </t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr"/>
+      <c r="M211" t="n">
+        <v>687</v>
+      </c>
+      <c r="N211" t="n">
+        <v>10</v>
+      </c>
+      <c r="O211" t="n">
+        <v>25</v>
+      </c>
+      <c r="P211" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q211" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="R211" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="S211" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="T211" t="n">
+        <v>1.63</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>213</v>
+      </c>
+      <c r="B212" t="n">
+        <v>38</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F212" t="n">
+        <v>19890</v>
+      </c>
+      <c r="G212" t="n">
+        <v>19890</v>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr"/>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr"/>
+      <c r="M212" t="n">
+        <v>0</v>
+      </c>
+      <c r="N212" t="n">
+        <v>0</v>
+      </c>
+      <c r="O212" t="n">
+        <v>0</v>
+      </c>
+      <c r="P212" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q212" t="n">
+        <v>0</v>
+      </c>
+      <c r="R212" t="n">
+        <v>0</v>
+      </c>
+      <c r="S212" t="n">
+        <v>0</v>
+      </c>
+      <c r="T212" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>214</v>
+      </c>
+      <c r="B213" t="n">
+        <v>37</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F213" t="n">
+        <v>7788</v>
+      </c>
+      <c r="G213" t="n">
+        <v>23673</v>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr"/>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr"/>
+      <c r="M213" t="n">
+        <v>0</v>
+      </c>
+      <c r="N213" t="n">
+        <v>0</v>
+      </c>
+      <c r="O213" t="n">
+        <v>0</v>
+      </c>
+      <c r="P213" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q213" t="n">
+        <v>0</v>
+      </c>
+      <c r="R213" t="n">
+        <v>0</v>
+      </c>
+      <c r="S213" t="n">
+        <v>0</v>
+      </c>
+      <c r="T213" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>215</v>
+      </c>
+      <c r="B214" t="n">
+        <v>37</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F214" t="n">
+        <v>26712</v>
+      </c>
+      <c r="G214" t="n">
+        <v>26712</v>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr"/>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr"/>
+      <c r="M214" t="n">
+        <v>0</v>
+      </c>
+      <c r="N214" t="n">
+        <v>0</v>
+      </c>
+      <c r="O214" t="n">
+        <v>0</v>
+      </c>
+      <c r="P214" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q214" t="n">
+        <v>0</v>
+      </c>
+      <c r="R214" t="n">
+        <v>0</v>
+      </c>
+      <c r="S214" t="n">
+        <v>0</v>
+      </c>
+      <c r="T214" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>216</v>
+      </c>
+      <c r="B215" t="n">
+        <v>36</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>10433</v>
+      </c>
+      <c r="G215" t="n">
+        <v>21174</v>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr"/>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr"/>
+      <c r="M215" t="n">
+        <v>0</v>
+      </c>
+      <c r="N215" t="n">
+        <v>0</v>
+      </c>
+      <c r="O215" t="n">
+        <v>0</v>
+      </c>
+      <c r="P215" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q215" t="n">
+        <v>0</v>
+      </c>
+      <c r="R215" t="n">
+        <v>0</v>
+      </c>
+      <c r="S215" t="n">
+        <v>0</v>
+      </c>
+      <c r="T215" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>217</v>
+      </c>
+      <c r="B216" t="n">
+        <v>36</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>21455</v>
+      </c>
+      <c r="G216" t="n">
+        <v>21455</v>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr"/>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr"/>
+      <c r="M216" t="n">
+        <v>0</v>
+      </c>
+      <c r="N216" t="n">
+        <v>0</v>
+      </c>
+      <c r="O216" t="n">
+        <v>0</v>
+      </c>
+      <c r="P216" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q216" t="n">
+        <v>0</v>
+      </c>
+      <c r="R216" t="n">
+        <v>0</v>
+      </c>
+      <c r="S216" t="n">
+        <v>0</v>
+      </c>
+      <c r="T216" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>218</v>
+      </c>
+      <c r="B217" t="n">
+        <v>36</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>9240</v>
+      </c>
+      <c r="G217" t="n">
+        <v>19876</v>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr"/>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr"/>
+      <c r="M217" t="n">
+        <v>0</v>
+      </c>
+      <c r="N217" t="n">
+        <v>0</v>
+      </c>
+      <c r="O217" t="n">
+        <v>0</v>
+      </c>
+      <c r="P217" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q217" t="n">
+        <v>0</v>
+      </c>
+      <c r="R217" t="n">
+        <v>0</v>
+      </c>
+      <c r="S217" t="n">
+        <v>0</v>
+      </c>
+      <c r="T217" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>219</v>
+      </c>
+      <c r="B218" t="n">
+        <v>37</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>25396</v>
+      </c>
+      <c r="G218" t="n">
+        <v>25396</v>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr"/>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr"/>
+      <c r="M218" t="n">
+        <v>0</v>
+      </c>
+      <c r="N218" t="n">
+        <v>0</v>
+      </c>
+      <c r="O218" t="n">
+        <v>0</v>
+      </c>
+      <c r="P218" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q218" t="n">
+        <v>0</v>
+      </c>
+      <c r="R218" t="n">
+        <v>0</v>
+      </c>
+      <c r="S218" t="n">
+        <v>0</v>
+      </c>
+      <c r="T218" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>220</v>
+      </c>
+      <c r="B219" t="n">
+        <v>37</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F219" t="n">
+        <v>5645</v>
+      </c>
+      <c r="G219" t="n">
+        <v>18249</v>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr"/>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr"/>
+      <c r="M219" t="n">
+        <v>0</v>
+      </c>
+      <c r="N219" t="n">
+        <v>0</v>
+      </c>
+      <c r="O219" t="n">
+        <v>0</v>
+      </c>
+      <c r="P219" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q219" t="n">
+        <v>0</v>
+      </c>
+      <c r="R219" t="n">
+        <v>0</v>
+      </c>
+      <c r="S219" t="n">
+        <v>0</v>
+      </c>
+      <c r="T219" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>221</v>
+      </c>
+      <c r="B220" t="n">
+        <v>38</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F220" t="n">
+        <v>20197</v>
+      </c>
+      <c r="G220" t="n">
+        <v>26581</v>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr"/>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr"/>
+      <c r="M220" t="n">
+        <v>0</v>
+      </c>
+      <c r="N220" t="n">
+        <v>0</v>
+      </c>
+      <c r="O220" t="n">
+        <v>0</v>
+      </c>
+      <c r="P220" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q220" t="n">
+        <v>0</v>
+      </c>
+      <c r="R220" t="n">
+        <v>0</v>
+      </c>
+      <c r="S220" t="n">
+        <v>0</v>
+      </c>
+      <c r="T220" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>222</v>
+      </c>
+      <c r="B221" t="n">
+        <v>38</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F221" t="n">
+        <v>10724</v>
+      </c>
+      <c r="G221" t="n">
+        <v>25251</v>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr"/>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>Bigot</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr"/>
+      <c r="M221" t="n">
+        <v>0</v>
+      </c>
+      <c r="N221" t="n">
+        <v>0</v>
+      </c>
+      <c r="O221" t="n">
+        <v>0</v>
+      </c>
+      <c r="P221" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q221" t="n">
+        <v>0</v>
+      </c>
+      <c r="R221" t="n">
+        <v>0</v>
+      </c>
+      <c r="S221" t="n">
+        <v>0</v>
+      </c>
+      <c r="T221" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>223</v>
+      </c>
+      <c r="B222" t="n">
+        <v>38</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F222" t="n">
+        <v>10724</v>
+      </c>
+      <c r="G222" t="n">
+        <v>16242</v>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr"/>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr"/>
+      <c r="M222" t="n">
+        <v>0</v>
+      </c>
+      <c r="N222" t="n">
+        <v>0</v>
+      </c>
+      <c r="O222" t="n">
+        <v>0</v>
+      </c>
+      <c r="P222" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q222" t="n">
+        <v>0</v>
+      </c>
+      <c r="R222" t="n">
+        <v>0</v>
+      </c>
+      <c r="S222" t="n">
+        <v>0</v>
+      </c>
+      <c r="T222" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>224</v>
+      </c>
+      <c r="B223" t="n">
+        <v>38</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F223" t="n">
+        <v>14850</v>
+      </c>
+      <c r="G223" t="n">
+        <v>28466</v>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr"/>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr"/>
+      <c r="M223" t="n">
+        <v>0</v>
+      </c>
+      <c r="N223" t="n">
+        <v>0</v>
+      </c>
+      <c r="O223" t="n">
+        <v>0</v>
+      </c>
+      <c r="P223" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q223" t="n">
+        <v>0</v>
+      </c>
+      <c r="R223" t="n">
+        <v>0</v>
+      </c>
+      <c r="S223" t="n">
+        <v>0</v>
+      </c>
+      <c r="T223" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>225</v>
+      </c>
+      <c r="B224" t="n">
+        <v>39</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F224" t="n">
+        <v>9326</v>
+      </c>
+      <c r="G224" t="n">
+        <v>37529</v>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr"/>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr"/>
+      <c r="M224" t="n">
+        <v>0</v>
+      </c>
+      <c r="N224" t="n">
+        <v>0</v>
+      </c>
+      <c r="O224" t="n">
+        <v>0</v>
+      </c>
+      <c r="P224" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q224" t="n">
+        <v>0</v>
+      </c>
+      <c r="R224" t="n">
+        <v>0</v>
+      </c>
+      <c r="S224" t="n">
+        <v>0</v>
+      </c>
+      <c r="T224" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>226</v>
+      </c>
+      <c r="B225" t="n">
+        <v>38</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Montdorensis</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F225" t="n">
+        <v>25290</v>
+      </c>
+      <c r="G225" t="n">
+        <v>41757</v>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr"/>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr"/>
+      <c r="M225" t="n">
+        <v>0</v>
+      </c>
+      <c r="N225" t="n">
+        <v>0</v>
+      </c>
+      <c r="O225" t="n">
+        <v>0</v>
+      </c>
+      <c r="P225" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q225" t="n">
+        <v>0</v>
+      </c>
+      <c r="R225" t="n">
+        <v>0</v>
+      </c>
+      <c r="S225" t="n">
+        <v>0</v>
+      </c>
+      <c r="T225" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>227</v>
+      </c>
+      <c r="B226" t="n">
+        <v>39</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Montdorensis</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F226" t="n">
+        <v>28883</v>
+      </c>
+      <c r="G226" t="n">
+        <v>29533</v>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr"/>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr"/>
+      <c r="M226" t="n">
+        <v>0</v>
+      </c>
+      <c r="N226" t="n">
+        <v>0</v>
+      </c>
+      <c r="O226" t="n">
+        <v>0</v>
+      </c>
+      <c r="P226" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q226" t="n">
+        <v>0</v>
+      </c>
+      <c r="R226" t="n">
+        <v>0</v>
+      </c>
+      <c r="S226" t="n">
+        <v>0</v>
+      </c>
+      <c r="T226" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>228</v>
+      </c>
+      <c r="B227" t="n">
+        <v>38</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Montdorensis</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F227" t="n">
+        <v>68050</v>
+      </c>
+      <c r="G227" t="n">
+        <v>68050</v>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr"/>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr"/>
+      <c r="M227" t="n">
+        <v>0</v>
+      </c>
+      <c r="N227" t="n">
+        <v>0</v>
+      </c>
+      <c r="O227" t="n">
+        <v>0</v>
+      </c>
+      <c r="P227" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q227" t="n">
+        <v>0</v>
+      </c>
+      <c r="R227" t="n">
+        <v>0</v>
+      </c>
+      <c r="S227" t="n">
+        <v>0</v>
+      </c>
+      <c r="T227" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>229</v>
+      </c>
+      <c r="B228" t="n">
+        <v>38</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Montdorensis</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F228" t="n">
+        <v>19184</v>
+      </c>
+      <c r="G228" t="n">
+        <v>61551</v>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr"/>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>S.A</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr"/>
+      <c r="M228" t="n">
+        <v>0</v>
+      </c>
+      <c r="N228" t="n">
+        <v>0</v>
+      </c>
+      <c r="O228" t="n">
+        <v>0</v>
+      </c>
+      <c r="P228" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q228" t="n">
+        <v>0</v>
+      </c>
+      <c r="R228" t="n">
+        <v>0</v>
+      </c>
+      <c r="S228" t="n">
+        <v>0</v>
+      </c>
+      <c r="T228" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>230</v>
+      </c>
+      <c r="B229" t="n">
+        <v>38</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Californicus</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F229" t="n">
+        <v>23442</v>
+      </c>
+      <c r="G229" t="n">
+        <v>23442</v>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr"/>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr"/>
+      <c r="M229" t="n">
+        <v>0</v>
+      </c>
+      <c r="N229" t="n">
+        <v>0</v>
+      </c>
+      <c r="O229" t="n">
+        <v>0</v>
+      </c>
+      <c r="P229" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q229" t="n">
+        <v>0</v>
+      </c>
+      <c r="R229" t="n">
+        <v>0</v>
+      </c>
+      <c r="S229" t="n">
+        <v>0</v>
+      </c>
+      <c r="T229" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>231</v>
+      </c>
+      <c r="B230" t="n">
+        <v>37</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Cucumeris</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F230" t="n">
+        <v>32188</v>
+      </c>
+      <c r="G230" t="n">
+        <v>34066</v>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr"/>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr"/>
+      <c r="M230" t="n">
+        <v>0</v>
+      </c>
+      <c r="N230" t="n">
+        <v>0</v>
+      </c>
+      <c r="O230" t="n">
+        <v>0</v>
+      </c>
+      <c r="P230" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q230" t="n">
+        <v>0</v>
+      </c>
+      <c r="R230" t="n">
+        <v>0</v>
+      </c>
+      <c r="S230" t="n">
+        <v>0</v>
+      </c>
+      <c r="T230" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>232</v>
+      </c>
+      <c r="B231" t="n">
+        <v>38</v>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Cucumeris</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F231" t="n">
+        <v>31715</v>
+      </c>
+      <c r="G231" t="n">
+        <v>34541</v>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr"/>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr"/>
+      <c r="M231" t="n">
+        <v>0</v>
+      </c>
+      <c r="N231" t="n">
+        <v>0</v>
+      </c>
+      <c r="O231" t="n">
+        <v>0</v>
+      </c>
+      <c r="P231" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q231" t="n">
+        <v>0</v>
+      </c>
+      <c r="R231" t="n">
+        <v>0</v>
+      </c>
+      <c r="S231" t="n">
+        <v>0</v>
+      </c>
+      <c r="T231" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>233</v>
+      </c>
+      <c r="B232" t="n">
+        <v>38</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Swirskii</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F232" t="n">
+        <v>22904</v>
+      </c>
+      <c r="G232" t="n">
+        <v>24464</v>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr"/>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>S.A</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr"/>
+      <c r="M232" t="n">
+        <v>0</v>
+      </c>
+      <c r="N232" t="n">
+        <v>0</v>
+      </c>
+      <c r="O232" t="n">
+        <v>0</v>
+      </c>
+      <c r="P232" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q232" t="n">
+        <v>0</v>
+      </c>
+      <c r="R232" t="n">
+        <v>0</v>
+      </c>
+      <c r="S232" t="n">
+        <v>0</v>
+      </c>
+      <c r="T232" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>234</v>
+      </c>
+      <c r="B233" t="n">
+        <v>38</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Swirskii</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F233" t="n">
+        <v>15817</v>
+      </c>
+      <c r="G233" t="n">
+        <v>30578</v>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr"/>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr"/>
+      <c r="M233" t="n">
+        <v>0</v>
+      </c>
+      <c r="N233" t="n">
+        <v>0</v>
+      </c>
+      <c r="O233" t="n">
+        <v>0</v>
+      </c>
+      <c r="P233" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>0</v>
+      </c>
+      <c r="R233" t="n">
+        <v>0</v>
+      </c>
+      <c r="S233" t="n">
+        <v>0</v>
+      </c>
+      <c r="T233" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>235</v>
+      </c>
+      <c r="B234" t="n">
+        <v>38</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Swirskii</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F234" t="n">
+        <v>25200</v>
+      </c>
+      <c r="G234" t="n">
+        <v>25200</v>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr"/>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr"/>
+      <c r="M234" t="n">
+        <v>0</v>
+      </c>
+      <c r="N234" t="n">
+        <v>0</v>
+      </c>
+      <c r="O234" t="n">
+        <v>0</v>
+      </c>
+      <c r="P234" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q234" t="n">
+        <v>0</v>
+      </c>
+      <c r="R234" t="n">
+        <v>0</v>
+      </c>
+      <c r="S234" t="n">
+        <v>0</v>
+      </c>
+      <c r="T234" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>236</v>
+      </c>
+      <c r="B235" t="n">
+        <v>36</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F235" t="n">
+        <v>55729</v>
+      </c>
+      <c r="G235" t="n">
+        <v>71309</v>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr"/>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr"/>
+      <c r="M235" t="n">
+        <v>0</v>
+      </c>
+      <c r="N235" t="n">
+        <v>0</v>
+      </c>
+      <c r="O235" t="n">
+        <v>0</v>
+      </c>
+      <c r="P235" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q235" t="n">
+        <v>0</v>
+      </c>
+      <c r="R235" t="n">
+        <v>0</v>
+      </c>
+      <c r="S235" t="n">
+        <v>0</v>
+      </c>
+      <c r="T235" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>237</v>
+      </c>
+      <c r="B236" t="n">
+        <v>37</v>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F236" t="n">
+        <v>30168</v>
+      </c>
+      <c r="G236" t="n">
+        <v>44979</v>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr"/>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr"/>
+      <c r="M236" t="n">
+        <v>0</v>
+      </c>
+      <c r="N236" t="n">
+        <v>0</v>
+      </c>
+      <c r="O236" t="n">
+        <v>0</v>
+      </c>
+      <c r="P236" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q236" t="n">
+        <v>0</v>
+      </c>
+      <c r="R236" t="n">
+        <v>0</v>
+      </c>
+      <c r="S236" t="n">
+        <v>0</v>
+      </c>
+      <c r="T236" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>238</v>
+      </c>
+      <c r="B237" t="n">
+        <v>38</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F237" t="n">
+        <v>25242</v>
+      </c>
+      <c r="G237" t="n">
+        <v>56191</v>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr"/>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr"/>
+      <c r="M237" t="n">
+        <v>0</v>
+      </c>
+      <c r="N237" t="n">
+        <v>0</v>
+      </c>
+      <c r="O237" t="n">
+        <v>0</v>
+      </c>
+      <c r="P237" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q237" t="n">
+        <v>0</v>
+      </c>
+      <c r="R237" t="n">
+        <v>0</v>
+      </c>
+      <c r="S237" t="n">
+        <v>0</v>
+      </c>
+      <c r="T237" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>239</v>
+      </c>
+      <c r="B238" t="n">
+        <v>36</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F238" t="n">
+        <v>351057</v>
+      </c>
+      <c r="G238" t="n">
+        <v>351057</v>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>250,000</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr"/>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>250,000</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>Sher</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr"/>
+      <c r="M238" t="n">
+        <v>0</v>
+      </c>
+      <c r="N238" t="n">
+        <v>0</v>
+      </c>
+      <c r="O238" t="n">
+        <v>0</v>
+      </c>
+      <c r="P238" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q238" t="n">
+        <v>0</v>
+      </c>
+      <c r="R238" t="n">
+        <v>0</v>
+      </c>
+      <c r="S238" t="n">
+        <v>0</v>
+      </c>
+      <c r="T238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>240</v>
+      </c>
+      <c r="B239" t="n">
+        <v>37</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F239" t="n">
+        <v>196363</v>
+      </c>
+      <c r="G239" t="n">
+        <v>331632</v>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>250,000</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr"/>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>250,000</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>Sher</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr"/>
+      <c r="M239" t="n">
+        <v>0</v>
+      </c>
+      <c r="N239" t="n">
+        <v>0</v>
+      </c>
+      <c r="O239" t="n">
+        <v>0</v>
+      </c>
+      <c r="P239" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q239" t="n">
+        <v>0</v>
+      </c>
+      <c r="R239" t="n">
+        <v>0</v>
+      </c>
+      <c r="S239" t="n">
+        <v>0</v>
+      </c>
+      <c r="T239" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>241</v>
+      </c>
+      <c r="B240" t="n">
+        <v>38</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="F240" t="n">
+        <v>171441</v>
+      </c>
+      <c r="G240" t="n">
+        <v>318284</v>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>250,000</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr"/>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>250,000</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>Sher</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr"/>
+      <c r="M240" t="n">
+        <v>0</v>
+      </c>
+      <c r="N240" t="n">
+        <v>0</v>
+      </c>
+      <c r="O240" t="n">
+        <v>0</v>
+      </c>
+      <c r="P240" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q240" t="n">
+        <v>0</v>
+      </c>
+      <c r="R240" t="n">
+        <v>0</v>
+      </c>
+      <c r="S240" t="n">
+        <v>0</v>
+      </c>
+      <c r="T240" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>242</v>
+      </c>
+      <c r="B241" t="n">
+        <v>36</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F241" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G241" t="n">
+        <v>73114</v>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>250,000</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr"/>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr"/>
+      <c r="M241" t="n">
+        <v>0</v>
+      </c>
+      <c r="N241" t="n">
+        <v>0</v>
+      </c>
+      <c r="O241" t="n">
+        <v>0</v>
+      </c>
+      <c r="P241" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q241" t="n">
+        <v>0</v>
+      </c>
+      <c r="R241" t="n">
+        <v>0</v>
+      </c>
+      <c r="S241" t="n">
+        <v>0</v>
+      </c>
+      <c r="T241" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>243</v>
+      </c>
+      <c r="B242" t="n">
+        <v>36</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F242" t="n">
+        <v>43600</v>
+      </c>
+      <c r="G242" t="n">
+        <v>43600</v>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr"/>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr"/>
+      <c r="M242" t="n">
+        <v>0</v>
+      </c>
+      <c r="N242" t="n">
+        <v>0</v>
+      </c>
+      <c r="O242" t="n">
+        <v>0</v>
+      </c>
+      <c r="P242" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q242" t="n">
+        <v>0</v>
+      </c>
+      <c r="R242" t="n">
+        <v>0</v>
+      </c>
+      <c r="S242" t="n">
+        <v>0</v>
+      </c>
+      <c r="T242" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>244</v>
+      </c>
+      <c r="B243" t="n">
+        <v>36</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F243" t="n">
+        <v>10663</v>
+      </c>
+      <c r="G243" t="n">
+        <v>45000</v>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr"/>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr"/>
+      <c r="M243" t="n">
+        <v>0</v>
+      </c>
+      <c r="N243" t="n">
+        <v>0</v>
+      </c>
+      <c r="O243" t="n">
+        <v>0</v>
+      </c>
+      <c r="P243" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q243" t="n">
+        <v>0</v>
+      </c>
+      <c r="R243" t="n">
+        <v>0</v>
+      </c>
+      <c r="S243" t="n">
+        <v>0</v>
+      </c>
+      <c r="T243" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>245</v>
+      </c>
+      <c r="B244" t="n">
+        <v>37</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F244" t="n">
+        <v>25752</v>
+      </c>
+      <c r="G244" t="n">
+        <v>25752</v>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr"/>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr"/>
+      <c r="M244" t="n">
+        <v>0</v>
+      </c>
+      <c r="N244" t="n">
+        <v>0</v>
+      </c>
+      <c r="O244" t="n">
+        <v>0</v>
+      </c>
+      <c r="P244" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q244" t="n">
+        <v>0</v>
+      </c>
+      <c r="R244" t="n">
+        <v>0</v>
+      </c>
+      <c r="S244" t="n">
+        <v>0</v>
+      </c>
+      <c r="T244" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>246</v>
+      </c>
+      <c r="B245" t="n">
+        <v>37</v>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F245" t="n">
+        <v>29274</v>
+      </c>
+      <c r="G245" t="n">
+        <v>42296</v>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr"/>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr"/>
+      <c r="M245" t="n">
+        <v>0</v>
+      </c>
+      <c r="N245" t="n">
+        <v>0</v>
+      </c>
+      <c r="O245" t="n">
+        <v>0</v>
+      </c>
+      <c r="P245" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q245" t="n">
+        <v>0</v>
+      </c>
+      <c r="R245" t="n">
+        <v>0</v>
+      </c>
+      <c r="S245" t="n">
+        <v>0</v>
+      </c>
+      <c r="T245" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>247</v>
+      </c>
+      <c r="B246" t="n">
+        <v>37</v>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Hypoaspis</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F246" t="n">
+        <v>9895</v>
+      </c>
+      <c r="G246" t="n">
+        <v>57004</v>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr"/>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>Other local customers</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr"/>
+      <c r="M246" t="n">
+        <v>0</v>
+      </c>
+      <c r="N246" t="n">
+        <v>0</v>
+      </c>
+      <c r="O246" t="n">
+        <v>0</v>
+      </c>
+      <c r="P246" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q246" t="n">
+        <v>0</v>
+      </c>
+      <c r="R246" t="n">
+        <v>0</v>
+      </c>
+      <c r="S246" t="n">
+        <v>0</v>
+      </c>
+      <c r="T246" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>